<commit_message>
Migrate Help & Support page: header, footer, blocks, styling
Content migration for the "help-and-support" template (index page):
- hero-support, cards-quicklink (horizontal carousel), app-promo,
  carousel-tips, accordion-faq (5 categories), cards-support parsers
  rewritten for the EDS-rendered DOM
- Navigation (header) with hamburger drawer + nav.plain.html
- Footer with app badges, gradient logo band, teal social chips, legal row
- Design: teal FAQ heading + pills, mint carousel, two-column FAQ layout,
  section spacing, local assets under content/images
- taqa-cleanup transformer now strips the global header/footer
- Local esbuild-free bundler (.bundle-helper.mjs) for this environment

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-help-and-support.report.xlsx
+++ b/tools/importer/reports/import-help-and-support.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="48">
   <si>
     <t>_reportFile</t>
   </si>
@@ -64,19 +64,22 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["carousel-hero","cards-quicklink","cards-quicklink","carousel-fare","cards-news","columns-appbanner","accordion-faq","columns-newsletter"]</t>
+    <t>["hero-support","cards-quicklink","app-promo","carousel-tips","accordion-faq","cards-support"]</t>
   </si>
   <si>
     <t>index</t>
   </si>
   <si>
-    <t>home-landing</t>
-  </si>
-  <si>
-    <t>2026-07-19T09:47:55.705Z</t>
-  </si>
-  <si>
-    <t>https://www.nileair.com/</t>
+    <t>help-and-support</t>
+  </si>
+  <si>
+    <t>2026-09-21T10:07:19.295Z</t>
+  </si>
+  <si>
+    <t>TAQA Distribution</t>
+  </si>
+  <si>
+    <t>https://main--demoenvironment--lmanning2.aem.live/addc/en-us/residential/help-and-support/transfer-and-removal-of-electricity-services</t>
   </si>
   <si>
     <t>nileair-holidays.report.json</t>
@@ -109,6 +112,24 @@
     <t>https://www.nileair.com/travelling-pets</t>
   </si>
   <si>
+    <t>addc/en-us/residential/overview.report.json</t>
+  </si>
+  <si>
+    <t>["hero-residential","cards-usp-overlay","cards-usp-overlay","cards-news"]</t>
+  </si>
+  <si>
+    <t>addc/en-us/residential/overview</t>
+  </si>
+  <si>
+    <t>residential</t>
+  </si>
+  <si>
+    <t>2026-09-17T05:56:42.554Z</t>
+  </si>
+  <si>
+    <t>https://taqadistribution.com/addc/en-us/residential/overview</t>
+  </si>
+  <si>
     <t>addc/en-us/business/help-and-support/certificates.report.json</t>
   </si>
   <si>
@@ -118,28 +139,22 @@
     <t>addc/en-us/business/help-and-support/certificates</t>
   </si>
   <si>
-    <t>help-and-support</t>
-  </si>
-  <si>
     <t>2026-09-16T08:55:32.399Z</t>
   </si>
   <si>
-    <t>TAQA Distribution</t>
-  </si>
-  <si>
     <t>https://taqadistribution.com/addc/en-us/business/help-and-support/certificates</t>
   </si>
   <si>
     <t>addc/en-us/residential/help-and-support/transfer-and-removal-of-electricity-services.report.json</t>
   </si>
   <si>
+    <t>[]</t>
+  </si>
+  <si>
     <t>addc/en-us/residential/help-and-support/transfer-and-removal-of-electricity-services</t>
   </si>
   <si>
-    <t>2026-09-16T08:55:44.447Z</t>
-  </si>
-  <si>
-    <t>https://taqadistribution.com/addc/en-us/residential/help-and-support/transfer-and-removal-of-electricity-services</t>
+    <t>2026-09-21T07:34:45.422Z</t>
   </si>
 </sst>
 </file>
@@ -528,7 +543,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -610,21 +625,21 @@
         <v>20</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="H3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
@@ -633,24 +648,24 @@
         <v>12</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
         <v>14</v>
       </c>
       <c r="H4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
@@ -659,36 +674,36 @@
         <v>12</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G5" t="s">
         <v>14</v>
       </c>
       <c r="H5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G6" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="H6" t="s">
         <v>38</v>
@@ -699,25 +714,51 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G7" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="H7" t="s">
-        <v>42</v>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>